<commit_message>
0.7.0 Fix cameraDevice, add performencaDateTime, make aiDevice and sectraStudyId optional
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-cautions-extension.xlsx
+++ b/docs/StructureDefinition-cautions-extension.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.0</t>
+    <t>0.7.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-03T09:57:13+01:00</t>
+    <t>2026-03-31T17:09:32+02:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
0.9.1 Add examination state diagram for append operation
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-cautions-extension.xlsx
+++ b/docs/StructureDefinition-cautions-extension.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.0</t>
+    <t>0.9.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-05T15:47:27+02:00</t>
+    <t>2026-06-08T15:50:57+02:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>